<commit_message>
Fix minor adjustments to main.html and main.js
</commit_message>
<xml_diff>
--- a/excel.xlsx
+++ b/excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\PROTRAINING\Notas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B802DC8-CA85-41B1-BBCD-BD89AF242EFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA4F427-C597-417D-BDF0-9658E726F826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="7" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VM" sheetId="11" state="hidden" r:id="rId1"/>
@@ -1559,34 +1559,38 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" pivotButton="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1598,13 +1602,9 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" pivotButton="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -1625,7 +1625,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Admin" refreshedDate="46206.395921064817" refreshedVersion="8" recordCount="1" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Admin" refreshedDate="46206.406901967595" refreshedVersion="8" recordCount="1" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:C320" sheet="Consolidado"/>
   </cacheSource>
@@ -1715,8 +1715,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000005000000}" name="CURSOSXESTUDIANTES 2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="G5:I8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000008000000}" name="CURSOSXESTUDIANTES 6" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="G20:I23" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1767,8 +1767,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000004000000}" name="CURSOSXESTUDIANTES 7" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A27:C30" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000D000000}" name="CURSOSXESTUDIANTES 13" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="A48:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1819,8 +1819,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000003000000}" name="CURSOSXESTUDIANTES 12" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="G41:I44" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000C000000}" name="CURSOSXESTUDIANTES 9" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="A34:C37" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1923,6 +1923,110 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000007000000}" name="CURSOSXESTUDIANTES" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000B000000}" name="CURSOSXESTUDIANTES 4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="G13:I16" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000001000000}" name="CURSOSXESTUDIANTES 8" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
   <location ref="G27:I30" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
@@ -1974,113 +2078,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000D000000}" name="CURSOSXESTUDIANTES 13" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A48:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000C000000}" name="CURSOSXESTUDIANTES 9" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A34:C37" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000B000000}" name="CURSOSXESTUDIANTES 4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="G13:I16" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000006000000}" name="CURSOSXESTUDIANTES 11" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="A41:C44" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -2131,6 +2131,58 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000005000000}" name="CURSOSXESTUDIANTES 2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="G5:I8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-00000A000000}" name="CURSOSXESTUDIANTES 10" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
   <location ref="G34:I37" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
@@ -2182,7 +2234,59 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000004000000}" name="CURSOSXESTUDIANTES 7" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="A27:C30" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
+  </dataFields>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000009000000}" name="CURSOSXESTUDIANTES 5" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
   <location ref="A20:C23" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
@@ -2234,113 +2338,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000008000000}" name="CURSOSXESTUDIANTES 6" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="G20:I23" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000007000000}" name="CURSOSXESTUDIANTES" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="3">
-    <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField name=" " dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name=" 2" axis="axisCol" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name=" " fld="1" subtotal="count" baseField="0"/>
-  </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000006000000}" name="CURSOSXESTUDIANTES 11" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A41:C44" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0E00-000003000000}" name="CURSOSXESTUDIANTES 12" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
+  <location ref="G41:I44" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField name="#VALUE!" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -2607,72 +2607,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="51" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="60" t="s">
         <v>266</v>
       </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="49"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="62"/>
     </row>
     <row r="2" spans="1:15" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="56" t="s">
+      <c r="C2" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="54" t="s">
+      <c r="D2" s="52" t="s">
         <v>267</v>
       </c>
-      <c r="E2" s="54" t="s">
+      <c r="E2" s="52" t="s">
         <v>268</v>
       </c>
-      <c r="F2" s="54" t="s">
+      <c r="F2" s="52" t="s">
         <v>269</v>
       </c>
-      <c r="G2" s="58" t="s">
+      <c r="G2" s="54" t="s">
         <v>236</v>
       </c>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
       <c r="J2" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="56" t="s">
         <v>270</v>
       </c>
-      <c r="L2" s="58" t="s">
+      <c r="L2" s="54" t="s">
         <v>271</v>
       </c>
-      <c r="M2" s="59"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="62" t="s">
+      <c r="M2" s="55"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="66" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
+      <c r="A3" s="64"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
       <c r="G3" s="1">
         <v>14</v>
       </c>
@@ -2685,7 +2685,7 @@
       <c r="J3" s="1">
         <v>11</v>
       </c>
-      <c r="K3" s="55"/>
+      <c r="K3" s="53"/>
       <c r="L3" s="1">
         <v>1</v>
       </c>
@@ -2695,7 +2695,7 @@
       <c r="N3" s="1">
         <v>3</v>
       </c>
-      <c r="O3" s="63"/>
+      <c r="O3" s="67"/>
     </row>
     <row r="4" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4"/>
@@ -20230,78 +20230,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="51" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="60" t="s">
         <v>277</v>
       </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="49"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="62"/>
     </row>
     <row r="2" spans="1:17" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="56" t="s">
+      <c r="C2" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="54" t="s">
+      <c r="D2" s="52" t="s">
         <v>267</v>
       </c>
-      <c r="E2" s="54" t="s">
+      <c r="E2" s="52" t="s">
         <v>268</v>
       </c>
-      <c r="F2" s="54" t="s">
+      <c r="F2" s="52" t="s">
         <v>269</v>
       </c>
-      <c r="G2" s="58" t="s">
+      <c r="G2" s="54" t="s">
         <v>236</v>
       </c>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="58" t="s">
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="54" t="s">
         <v>237</v>
       </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="61" t="s">
+      <c r="K2" s="55"/>
+      <c r="L2" s="56" t="s">
         <v>270</v>
       </c>
-      <c r="M2" s="61" t="s">
+      <c r="M2" s="56" t="s">
         <v>278</v>
       </c>
-      <c r="N2" s="58" t="s">
+      <c r="N2" s="54" t="s">
         <v>271</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="62" t="s">
+      <c r="O2" s="55"/>
+      <c r="P2" s="57"/>
+      <c r="Q2" s="66" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="53"/>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
+      <c r="A3" s="64"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
       <c r="G3" s="1">
         <v>14</v>
       </c>
@@ -20317,8 +20317,8 @@
       <c r="K3" s="1">
         <v>18</v>
       </c>
-      <c r="L3" s="55"/>
-      <c r="M3" s="55"/>
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
       <c r="N3" s="1">
         <v>1</v>
       </c>
@@ -20328,7 +20328,7 @@
       <c r="P3" s="1">
         <v>3</v>
       </c>
-      <c r="Q3" s="63"/>
+      <c r="Q3" s="67"/>
     </row>
     <row r="4" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4"/>
@@ -37445,34 +37445,34 @@
   <sheetFormatPr defaultColWidth="10.07421875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="47" t="s">
         <v>284</v>
       </c>
-      <c r="B1" s="66" t="s">
+      <c r="B1" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C1" s="67"/>
+      <c r="C1" s="48"/>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C2" s="69" t="s">
+      <c r="C2" s="50" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="71"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="72"/>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B4" s="73"/>
@@ -37496,112 +37496,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="69" t="s">
         <v>285</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="64" t="s">
+      <c r="A4" s="68" t="s">
         <v>286</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
-      <c r="G4" s="64" t="s">
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="57"/>
+      <c r="G4" s="68" t="s">
         <v>183</v>
       </c>
-      <c r="H4" s="59"/>
-      <c r="I4" s="60"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="57"/>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="66" t="s">
+      <c r="A5" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C5" s="67"/>
+      <c r="C5" s="48"/>
       <c r="D5" s="42"/>
       <c r="E5" s="43"/>
-      <c r="G5" s="66" t="s">
+      <c r="G5" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H5" s="66" t="s">
+      <c r="H5" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I5" s="67"/>
+      <c r="I5" s="48"/>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="68" t="s">
+      <c r="B6" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="50" t="s">
         <v>299</v>
       </c>
       <c r="D6" s="44"/>
       <c r="E6" s="44"/>
-      <c r="G6" s="66" t="s">
+      <c r="G6" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H6" s="68" t="s">
+      <c r="H6" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I6" s="69" t="s">
+      <c r="I6" s="50" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="68" t="s">
+      <c r="A7" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="71"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="72"/>
       <c r="D7" s="44"/>
       <c r="E7" s="44"/>
-      <c r="G7" s="68" t="s">
+      <c r="G7" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H7" s="70"/>
-      <c r="I7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="72"/>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="72" t="s">
+      <c r="A8" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B8" s="73"/>
       <c r="C8" s="74"/>
       <c r="D8" s="44"/>
       <c r="E8" s="44"/>
-      <c r="G8" s="72" t="s">
+      <c r="G8" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H8" s="73"/>
@@ -37611,90 +37611,90 @@
       <c r="F11" s="45"/>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="68" t="s">
         <v>154</v>
       </c>
-      <c r="B12" s="59"/>
-      <c r="C12" s="59"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
-      <c r="G12" s="64" t="s">
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="57"/>
+      <c r="G12" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="60"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="57"/>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="66" t="s">
+      <c r="A13" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B13" s="66" t="s">
+      <c r="B13" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C13" s="67"/>
+      <c r="C13" s="48"/>
       <c r="D13" s="42"/>
       <c r="E13" s="43"/>
-      <c r="G13" s="66" t="s">
+      <c r="G13" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H13" s="66" t="s">
+      <c r="H13" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I13" s="67"/>
+      <c r="I13" s="48"/>
       <c r="J13" s="42"/>
       <c r="K13" s="43"/>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="66" t="s">
+      <c r="A14" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B14" s="68" t="s">
+      <c r="B14" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C14" s="69" t="s">
+      <c r="C14" s="50" t="s">
         <v>299</v>
       </c>
       <c r="D14" s="44"/>
       <c r="E14" s="44"/>
-      <c r="G14" s="66" t="s">
+      <c r="G14" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H14" s="68" t="s">
+      <c r="H14" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I14" s="69" t="s">
+      <c r="I14" s="50" t="s">
         <v>299</v>
       </c>
       <c r="J14" s="44"/>
       <c r="K14" s="44"/>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B15" s="70"/>
-      <c r="C15" s="71"/>
+      <c r="B15" s="71"/>
+      <c r="C15" s="72"/>
       <c r="D15" s="44"/>
       <c r="E15" s="44"/>
-      <c r="G15" s="68" t="s">
+      <c r="G15" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H15" s="70"/>
-      <c r="I15" s="71"/>
+      <c r="H15" s="71"/>
+      <c r="I15" s="72"/>
       <c r="J15" s="44"/>
       <c r="K15" s="44"/>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="72" t="s">
+      <c r="A16" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B16" s="73"/>
       <c r="C16" s="74"/>
       <c r="D16" s="44"/>
       <c r="E16" s="44"/>
-      <c r="G16" s="72" t="s">
+      <c r="G16" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H16" s="73"/>
@@ -37703,87 +37703,87 @@
       <c r="K16" s="44"/>
     </row>
     <row r="19" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="64" t="s">
+      <c r="A19" s="68" t="s">
         <v>195</v>
       </c>
-      <c r="B19" s="59"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="60"/>
-      <c r="G19" s="64" t="s">
+      <c r="B19" s="55"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="57"/>
+      <c r="G19" s="68" t="s">
         <v>254</v>
       </c>
-      <c r="H19" s="59"/>
-      <c r="I19" s="59"/>
-      <c r="J19" s="60"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="55"/>
+      <c r="J19" s="57"/>
       <c r="K19" s="45"/>
     </row>
     <row r="20" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="66" t="s">
+      <c r="A20" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B20" s="66" t="s">
+      <c r="B20" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C20" s="67"/>
+      <c r="C20" s="48"/>
       <c r="D20" s="42"/>
       <c r="E20" s="43"/>
-      <c r="G20" s="66" t="s">
+      <c r="G20" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H20" s="66" t="s">
+      <c r="H20" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I20" s="67"/>
+      <c r="I20" s="48"/>
       <c r="J20" s="43"/>
     </row>
     <row r="21" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B21" s="68" t="s">
+      <c r="B21" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C21" s="69" t="s">
+      <c r="C21" s="50" t="s">
         <v>299</v>
       </c>
       <c r="D21" s="44"/>
       <c r="E21" s="44"/>
-      <c r="G21" s="66" t="s">
+      <c r="G21" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H21" s="68" t="s">
+      <c r="H21" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I21" s="69" t="s">
+      <c r="I21" s="50" t="s">
         <v>299</v>
       </c>
       <c r="J21" s="44"/>
     </row>
     <row r="22" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="68" t="s">
+      <c r="A22" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B22" s="70"/>
-      <c r="C22" s="71"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="72"/>
       <c r="D22" s="44"/>
       <c r="E22" s="44"/>
-      <c r="G22" s="68" t="s">
+      <c r="G22" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H22" s="70"/>
-      <c r="I22" s="71"/>
+      <c r="H22" s="71"/>
+      <c r="I22" s="72"/>
       <c r="J22" s="44"/>
     </row>
     <row r="23" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="72" t="s">
+      <c r="A23" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B23" s="73"/>
       <c r="C23" s="74"/>
       <c r="D23" s="44"/>
       <c r="E23" s="44"/>
-      <c r="G23" s="72" t="s">
+      <c r="G23" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H23" s="73"/>
@@ -37791,79 +37791,79 @@
       <c r="J23" s="44"/>
     </row>
     <row r="26" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="64" t="s">
+      <c r="A26" s="68" t="s">
         <v>287</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="60"/>
+      <c r="B26" s="55"/>
+      <c r="C26" s="57"/>
       <c r="D26" s="45"/>
       <c r="E26" s="45"/>
-      <c r="G26" s="64" t="s">
+      <c r="G26" s="68" t="s">
         <v>288</v>
       </c>
-      <c r="H26" s="59"/>
-      <c r="I26" s="59"/>
-      <c r="J26" s="60"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="57"/>
       <c r="K26" s="45"/>
     </row>
     <row r="27" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B27" s="66" t="s">
+      <c r="B27" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C27" s="67"/>
-      <c r="G27" s="66" t="s">
+      <c r="C27" s="48"/>
+      <c r="G27" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H27" s="66" t="s">
+      <c r="H27" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I27" s="67"/>
+      <c r="I27" s="48"/>
       <c r="J27" s="43"/>
     </row>
     <row r="28" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B28" s="68" t="s">
+      <c r="B28" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C28" s="69" t="s">
+      <c r="C28" s="50" t="s">
         <v>299</v>
       </c>
-      <c r="G28" s="66" t="s">
+      <c r="G28" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H28" s="68" t="s">
+      <c r="H28" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I28" s="69" t="s">
+      <c r="I28" s="50" t="s">
         <v>299</v>
       </c>
       <c r="J28" s="44"/>
     </row>
     <row r="29" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="68" t="s">
+      <c r="A29" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B29" s="70"/>
-      <c r="C29" s="71"/>
-      <c r="G29" s="68" t="s">
+      <c r="B29" s="71"/>
+      <c r="C29" s="72"/>
+      <c r="G29" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H29" s="70"/>
-      <c r="I29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="72"/>
       <c r="J29" s="44"/>
     </row>
     <row r="30" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="72" t="s">
+      <c r="A30" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B30" s="73"/>
       <c r="C30" s="74"/>
-      <c r="G30" s="72" t="s">
+      <c r="G30" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H30" s="73"/>
@@ -37871,90 +37871,90 @@
       <c r="J30" s="44"/>
     </row>
     <row r="33" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="64" t="s">
+      <c r="A33" s="68" t="s">
         <v>132</v>
       </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="60"/>
-      <c r="G33" s="64" t="s">
+      <c r="B33" s="55"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="57"/>
+      <c r="G33" s="68" t="s">
         <v>235</v>
       </c>
-      <c r="H33" s="59"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="59"/>
-      <c r="K33" s="60"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="55"/>
+      <c r="J33" s="55"/>
+      <c r="K33" s="57"/>
     </row>
     <row r="34" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B34" s="66" t="s">
+      <c r="B34" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C34" s="67"/>
+      <c r="C34" s="48"/>
       <c r="D34" s="42"/>
       <c r="E34" s="43"/>
-      <c r="G34" s="66" t="s">
+      <c r="G34" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H34" s="66" t="s">
+      <c r="H34" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I34" s="67"/>
+      <c r="I34" s="48"/>
       <c r="J34" s="42"/>
       <c r="K34" s="43"/>
     </row>
     <row r="35" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="66" t="s">
+      <c r="A35" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B35" s="68" t="s">
+      <c r="B35" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C35" s="69" t="s">
+      <c r="C35" s="50" t="s">
         <v>299</v>
       </c>
       <c r="D35" s="44"/>
       <c r="E35" s="44"/>
-      <c r="G35" s="66" t="s">
+      <c r="G35" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H35" s="68" t="s">
+      <c r="H35" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I35" s="69" t="s">
+      <c r="I35" s="50" t="s">
         <v>299</v>
       </c>
       <c r="J35" s="44"/>
       <c r="K35" s="44"/>
     </row>
     <row r="36" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="68" t="s">
+      <c r="A36" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B36" s="70"/>
-      <c r="C36" s="71"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="72"/>
       <c r="D36" s="44"/>
       <c r="E36" s="44"/>
-      <c r="G36" s="68" t="s">
+      <c r="G36" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H36" s="70"/>
-      <c r="I36" s="71"/>
+      <c r="H36" s="71"/>
+      <c r="I36" s="72"/>
       <c r="J36" s="44"/>
       <c r="K36" s="44"/>
     </row>
     <row r="37" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A37" s="72" t="s">
+      <c r="A37" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B37" s="73"/>
       <c r="C37" s="74"/>
       <c r="D37" s="44"/>
       <c r="E37" s="44"/>
-      <c r="G37" s="72" t="s">
+      <c r="G37" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H37" s="73"/>
@@ -37963,127 +37963,127 @@
       <c r="K37" s="44"/>
     </row>
     <row r="40" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="64" t="s">
+      <c r="A40" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="B40" s="59"/>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="60"/>
-      <c r="G40" s="64" t="s">
+      <c r="B40" s="55"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="57"/>
+      <c r="G40" s="68" t="s">
         <v>188</v>
       </c>
-      <c r="H40" s="59"/>
-      <c r="I40" s="60"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="57"/>
       <c r="J40" s="45"/>
       <c r="K40" s="45"/>
     </row>
     <row r="41" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="66" t="s">
+      <c r="A41" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B41" s="66" t="s">
+      <c r="B41" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C41" s="67"/>
+      <c r="C41" s="48"/>
       <c r="D41" s="42"/>
       <c r="E41" s="43"/>
-      <c r="G41" s="66" t="s">
+      <c r="G41" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="H41" s="66" t="s">
+      <c r="H41" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="I41" s="67"/>
+      <c r="I41" s="48"/>
     </row>
     <row r="42" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="66" t="s">
+      <c r="A42" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B42" s="68" t="s">
+      <c r="B42" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C42" s="69" t="s">
+      <c r="C42" s="50" t="s">
         <v>299</v>
       </c>
       <c r="D42" s="44"/>
       <c r="E42" s="44"/>
-      <c r="G42" s="66" t="s">
+      <c r="G42" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="H42" s="68" t="s">
+      <c r="H42" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="I42" s="69" t="s">
+      <c r="I42" s="50" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="68" t="s">
+      <c r="A43" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B43" s="70"/>
-      <c r="C43" s="71"/>
+      <c r="B43" s="71"/>
+      <c r="C43" s="72"/>
       <c r="D43" s="44"/>
       <c r="E43" s="44"/>
-      <c r="G43" s="68" t="s">
+      <c r="G43" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="H43" s="70"/>
-      <c r="I43" s="71"/>
+      <c r="H43" s="71"/>
+      <c r="I43" s="72"/>
     </row>
     <row r="44" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="72" t="s">
+      <c r="A44" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B44" s="73"/>
       <c r="C44" s="74"/>
       <c r="D44" s="44"/>
       <c r="E44" s="44"/>
-      <c r="G44" s="72" t="s">
+      <c r="G44" s="51" t="s">
         <v>299</v>
       </c>
       <c r="H44" s="73"/>
       <c r="I44" s="74"/>
     </row>
     <row r="47" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="68" t="s">
         <v>277</v>
       </c>
-      <c r="B47" s="59"/>
-      <c r="C47" s="60"/>
+      <c r="B47" s="55"/>
+      <c r="C47" s="57"/>
       <c r="D47" s="45"/>
       <c r="E47" s="45"/>
     </row>
     <row r="48" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A48" s="66" t="s">
+      <c r="A48" s="47" t="s">
         <v>187</v>
       </c>
-      <c r="B48" s="66" t="s">
+      <c r="B48" s="47" t="s">
         <v>296</v>
       </c>
-      <c r="C48" s="67"/>
+      <c r="C48" s="48"/>
     </row>
     <row r="49" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A49" s="66" t="s">
+      <c r="A49" s="47" t="s">
         <v>297</v>
       </c>
-      <c r="B49" s="68" t="s">
+      <c r="B49" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="C49" s="69" t="s">
+      <c r="C49" s="50" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A50" s="68" t="s">
+      <c r="A50" s="49" t="s">
         <v>298</v>
       </c>
-      <c r="B50" s="70"/>
-      <c r="C50" s="71"/>
+      <c r="B50" s="71"/>
+      <c r="C50" s="72"/>
     </row>
     <row r="51" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A51" s="72" t="s">
+      <c r="A51" s="51" t="s">
         <v>299</v>
       </c>
       <c r="B51" s="73"/>

</xml_diff>